<commit_message>
Update Knockout Stage Placement.xlsx
</commit_message>
<xml_diff>
--- a/Knockout Stage Placement.xlsx
+++ b/Knockout Stage Placement.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://dbschenker-my.sharepoint.com/personal/muhammadfarhan_wajdi_dbschenker_com/Documents/Documents/Github/Worldcup-Web/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8938264A-B6B4-406F-9CEC-DC1B93BD7EBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="8_{8938264A-B6B4-406F-9CEC-DC1B93BD7EBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{427C45CF-19E6-453D-9BB0-E6CC90EFADF7}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{C0B98A6E-9977-4E06-AD99-FBD3912880A2}"/>
   </bookViews>
@@ -654,9 +654,7 @@
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
-      <c r="E7" s="1" t="s">
-        <v>12</v>
-      </c>
+      <c r="E7" s="1"/>
       <c r="F7" s="1"/>
       <c r="G7" s="1"/>
       <c r="H7" s="1"/>
@@ -701,6 +699,9 @@
       <c r="D10" s="1" t="s">
         <v>29</v>
       </c>
+      <c r="E10" s="1" t="s">
+        <v>12</v>
+      </c>
       <c r="F10" s="1" t="s">
         <v>30</v>
       </c>
@@ -730,6 +731,9 @@
       </c>
       <c r="C12" s="1"/>
       <c r="D12" s="1"/>
+      <c r="E12" s="1" t="s">
+        <v>14</v>
+      </c>
       <c r="F12" s="1"/>
       <c r="G12" s="1"/>
       <c r="H12" s="1" t="s">
@@ -744,9 +748,7 @@
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>
       <c r="D13" s="1"/>
-      <c r="E13" s="1" t="s">
-        <v>14</v>
-      </c>
+      <c r="E13" s="1"/>
       <c r="F13" s="1"/>
       <c r="G13" s="1"/>
       <c r="H13" s="1"/>

</xml_diff>